<commit_message>
Add live animals to the product-family questionnaire
New visible "בעלי חיים" checkbox, distinct from the existing "מוצרים מן החי" (products of animal origin). Maps as a forced single-candidate selection to a new canonical matrix row (food-and-beverages-08) that reuses the existing agriculture/Veterinary Services signal, professional routing, CTA, and limitation -- no new question, no new professional category. 61 matrix rows, 1365/1365 frontend tests, 26/26 browser-acceptance runs. Backend unchanged.
</commit_message>
<xml_diff>
--- a/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
+++ b/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3607,6 +3607,53 @@
         </is>
       </c>
       <c r="L61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>מזון ומשקאות</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>בעלי חיים</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Add animal feed to the product-family questionnaire
New visible "מזון לבעלי חיים" checkbox, distinct from live animals, products of animal origin, and non-food pet products. Maps as a forced single-candidate selection to a new canonical matrix row (food-and-beverages-09) that reuses the existing agriculture/Veterinary Services signal, professional routing, CTA, and limitation -- no new question, no new professional category. Corrects the one misrouted "מזון לחיות מחמד" alias off the general pet-products row. 62 matrix rows, 1408/1408 frontend tests, 54/54 browser-acceptance runs. Backend unchanged.
</commit_message>
<xml_diff>
--- a/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
+++ b/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3650,6 +3650,53 @@
         </is>
       </c>
       <c r="K62" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>מזון ומשקאות</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>מזון לבעלי חיים</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
         <is>
           <t>חסר</t>
         </is>

</xml_diff>

<commit_message>
Add approved guidance for additional product families
Implements seven product-owner-approved product-family directions:
drones, non-food pet equipment/products, hand tools, packaging
products, paper and printed products, non-apparel textile products,
and glass and ceramic products. Reuses the existing family-selection,
matrix, guidance, and detailed-rule architecture throughout -- no new
question, professional category, or result state.

11 new canonical rows, 5 alias-only extensions to existing rows, one
corrected workbook signal (non-food pet products), and 3 alias/
substring collision fixes found and resolved during this pass's own
testing.
</commit_message>
<xml_diff>
--- a/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
+++ b/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לבדוק</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -3697,6 +3697,523 @@
         </is>
       </c>
       <c r="K63" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>חשמל ואלקטרוניקה</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>רחפן</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>בנייה ותעשייה</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>כלי עבודה ידניים</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>מוצרי צריכה נוספים</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>קרטון לאריזה</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>בנייה ותעשייה</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>קופסת עץ לאריזה</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>מוצרי צריכה נוספים</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>נייר ומוצרי דפוס</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>טקסטיל וריהוט</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>שטיחים</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>טקסטיל וריהוט</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>שמיכה רגילה</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ילדים ותינוקות</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>מחזיק מוצץ</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ילדים ותינוקות</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>מנשא לתינוק</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>טקסטיל וריהוט</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>מוצרי טקסטיל ביתיים</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>בנייה ותעשייה</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>זכוכית בטיחות לבניין</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
         <is>
           <t>חסר</t>
         </is>

</xml_diff>

<commit_message>
Add approved guidance for drones, packaging, paper, textiles, and related products
* Add approved guidance for additional product families

Implements seven product-owner-approved product-family directions:
drones, non-food pet equipment/products, hand tools, packaging
products, paper and printed products, non-apparel textile products,
and glass and ceramic products. Reuses the existing family-selection,
matrix, guidance, and detailed-rule architecture throughout -- no new
question, professional category, or result state.

11 new canonical rows, 5 alias-only extensions to existing rows, one
corrected workbook signal (non-food pet products), and 3 alias/
substring collision fixes found and resolved during this pass's own
testing.

* Refresh Wave 3 browser acceptance artifacts (final validation, 76/76)

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
+++ b/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לבדוק</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -3697,6 +3697,523 @@
         </is>
       </c>
       <c r="K63" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>חשמל ואלקטרוניקה</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>רחפן</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>בנייה ותעשייה</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>כלי עבודה ידניים</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>מוצרי צריכה נוספים</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>קרטון לאריזה</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>בנייה ותעשייה</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>קופסת עץ לאריזה</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>מוצרי צריכה נוספים</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>נייר ומוצרי דפוס</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>טקסטיל וריהוט</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>שטיחים</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>טקסטיל וריהוט</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>שמיכה רגילה</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ילדים ותינוקות</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>מחזיק מוצץ</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ילדים ותינוקות</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>מנשא לתינוק</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>טקסטיל וריהוט</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>מוצרי טקסטיל ביתיים</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>בנייה ותעשייה</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>זכוכית בטיחות לבניין</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
         <is>
           <t>חסר</t>
         </is>

</xml_diff>